<commit_message>
before the new curve
</commit_message>
<xml_diff>
--- a/Output/17072026_Accolade - KPI V1.14.xlsx
+++ b/Output/17072026_Accolade - KPI V1.14.xlsx
@@ -23212,10 +23212,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="54" customWidth="1" style="36" min="1" max="1"/>
+    <col width="55" customWidth="1" style="36" min="1" max="1"/>
     <col width="26" customWidth="1" style="36" min="2" max="2"/>
     <col width="26" customWidth="1" style="36" min="3" max="3"/>
     <col width="25" customWidth="1" style="36" min="4" max="4"/>
@@ -23232,449 +23232,487 @@
     <row r="3">
       <c r="A3" s="40" t="inlineStr">
         <is>
-          <t>Portefeuille</t>
+          <t>KPI issus de la feuille source</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="41" t="inlineStr">
         <is>
-          <t>Total pp non radiés</t>
+          <t>KPI 1 — Nouvelles souscriptions Accolade depuis 01/01/2024</t>
         </is>
       </c>
       <c r="B4" s="42" t="n">
-        <v>4101027</v>
+        <v>3580988</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="41" t="inlineStr">
         <is>
-          <t>Total pp à date</t>
+          <t>KPI 2 — Résiliations Accolade toutes dates</t>
         </is>
       </c>
       <c r="B5" s="42" t="n">
-        <v>4086120</v>
+        <v>544129</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="41" t="inlineStr">
         <is>
-          <t>Taux de radiation global</t>
-        </is>
-      </c>
-      <c r="B6" s="43" t="n">
-        <v>0.003634943149606184</v>
+          <t>KPI 2 Bis — Résiliations Accolade depuis 01/01/2024</t>
+        </is>
+      </c>
+      <c r="B6" s="42" t="n">
+        <v>490383</v>
       </c>
     </row>
     <row r="7"/>
     <row r="8">
       <c r="A8" s="40" t="inlineStr">
         <is>
-          <t>Qualité des données — Déphasages AI / KPEP (KPI 8)</t>
+          <t>Portefeuille</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="44" t="inlineStr">
-        <is>
-          <t>Indicateur</t>
-        </is>
-      </c>
-      <c r="B9" s="44" t="inlineStr">
-        <is>
-          <t>Nb déphasages</t>
-        </is>
-      </c>
-      <c r="C9" s="44" t="inlineStr">
-        <is>
-          <t>% portefeuille ASSURE</t>
-        </is>
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>Total pp non radiés</t>
+        </is>
+      </c>
+      <c r="B9" s="42" t="n">
+        <v>4101027</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="41" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="B10" s="45" t="n">
-        <v>20386</v>
-      </c>
-      <c r="C10" s="46" t="n">
-        <v>0.006363035092204081</v>
+          <t>Total pp à date</t>
+        </is>
+      </c>
+      <c r="B10" s="42" t="n">
+        <v>4086120</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="41" t="inlineStr">
         <is>
-          <t>Téléphone PORT</t>
-        </is>
-      </c>
-      <c r="B11" s="45" t="n">
-        <v>70995</v>
-      </c>
-      <c r="C11" s="46" t="n">
-        <v>0.0221595053650068</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="41" t="inlineStr">
-        <is>
-          <t>Téléphone TELP</t>
-        </is>
-      </c>
-      <c r="B12" s="45" t="n">
-        <v>5200</v>
-      </c>
-      <c r="C12" s="46" t="n">
-        <v>0.001623063988985638</v>
-      </c>
-    </row>
+          <t>Taux de radiation global</t>
+        </is>
+      </c>
+      <c r="B11" s="43" t="n">
+        <v>0.003634943149606184</v>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
-      <c r="A13" s="47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Total téléphone</t>
-        </is>
-      </c>
-      <c r="B13" s="48" t="n">
-        <v>76195</v>
-      </c>
-      <c r="C13" s="49" t="n">
-        <v>0.02378256935399244</v>
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>Qualité des données — Déphasages AI / KPEP (KPI 8)</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="41" t="inlineStr">
-        <is>
-          <t>Date de naissance</t>
-        </is>
-      </c>
-      <c r="B14" s="45" t="n">
-        <v>459</v>
-      </c>
-      <c r="C14" s="46" t="n">
-        <v>0.0001432666097970015</v>
+      <c r="A14" s="44" t="inlineStr">
+        <is>
+          <t>Indicateur</t>
+        </is>
+      </c>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t>Nb déphasages</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="inlineStr">
+        <is>
+          <t>% portefeuille ASSURE</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="41" t="inlineStr">
         <is>
-          <t>Date de décès</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="B15" s="45" t="n">
-        <v>3754</v>
+        <v>20386</v>
       </c>
       <c r="C15" s="46" t="n">
-        <v>0.001171727348971555</v>
+        <v>0.006363035092204081</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="41" t="inlineStr">
         <is>
-          <t>Adresses</t>
+          <t>Téléphone PORT</t>
         </is>
       </c>
       <c r="B16" s="45" t="n">
-        <v>83598</v>
+        <v>70995</v>
       </c>
       <c r="C16" s="46" t="n">
-        <v>0.02609325064446565</v>
-      </c>
-    </row>
-    <row r="17"/>
+        <v>0.0221595053650068</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
+          <t>Téléphone TELP</t>
+        </is>
+      </c>
+      <c r="B17" s="45" t="n">
+        <v>5200</v>
+      </c>
+      <c r="C17" s="46" t="n">
+        <v>0.001623063988985638</v>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="40" t="inlineStr">
-        <is>
-          <t>Résiliations</t>
-        </is>
+      <c r="A18" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Total téléphone</t>
+        </is>
+      </c>
+      <c r="B18" s="48" t="n">
+        <v>76195</v>
+      </c>
+      <c r="C18" s="49" t="n">
+        <v>0.02378256935399244</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="41" t="inlineStr">
         <is>
-          <t>Total résiliations</t>
-        </is>
-      </c>
-      <c r="B19" s="42" t="n">
-        <v>402283</v>
+          <t>Date de naissance</t>
+        </is>
+      </c>
+      <c r="B19" s="45" t="n">
+        <v>459</v>
+      </c>
+      <c r="C19" s="46" t="n">
+        <v>0.0001432666097970015</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="41" t="inlineStr">
         <is>
-          <t>Motif dominant</t>
-        </is>
-      </c>
-      <c r="B20" s="50" t="inlineStr">
-        <is>
-          <t>ANNUL</t>
-        </is>
+          <t>Date de décès</t>
+        </is>
+      </c>
+      <c r="B20" s="45" t="n">
+        <v>3754</v>
+      </c>
+      <c r="C20" s="46" t="n">
+        <v>0.001171727348971555</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="41" t="inlineStr">
         <is>
-          <t>Part du motif dominant</t>
-        </is>
-      </c>
-      <c r="B21" s="43" t="n">
-        <v>0.6324328892844092</v>
+          <t>Adresses</t>
+        </is>
+      </c>
+      <c r="B21" s="45" t="n">
+        <v>83598</v>
+      </c>
+      <c r="C21" s="46" t="n">
+        <v>0.02609325064446565</v>
       </c>
     </row>
     <row r="22"/>
     <row r="23">
       <c r="A23" s="40" t="inlineStr">
         <is>
-          <t>Top 3 offres ASSURE (pp non radiés)</t>
+          <t>Résiliations</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="41" t="inlineStr">
         <is>
-          <t>MESMEN001</t>
+          <t>Total résiliations</t>
         </is>
       </c>
       <c r="B24" s="42" t="n">
-        <v>1213928</v>
+        <v>402283</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="41" t="inlineStr">
         <is>
-          <t>INMMSPRET1</t>
-        </is>
-      </c>
-      <c r="B25" s="42" t="n">
-        <v>785885</v>
+          <t>Motif dominant</t>
+        </is>
+      </c>
+      <c r="B25" s="50" t="inlineStr">
+        <is>
+          <t>ANNUL</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="41" t="inlineStr">
         <is>
-          <t>INPPREVIND</t>
-        </is>
-      </c>
-      <c r="B26" s="42" t="n">
-        <v>691892</v>
+          <t>Part du motif dominant</t>
+        </is>
+      </c>
+      <c r="B26" s="43" t="n">
+        <v>0.6324328892844092</v>
       </c>
     </row>
     <row r="27"/>
     <row r="28">
       <c r="A28" s="40" t="inlineStr">
         <is>
-          <t>Fidélité par tranche d'âge</t>
+          <t>Top 3 offres ASSURE (pp non radiés)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="41" t="inlineStr">
         <is>
-          <t>Tranche la plus fidèle</t>
-        </is>
-      </c>
-      <c r="B29" s="50" t="inlineStr">
-        <is>
-          <t>Plus de 80 ans</t>
-        </is>
+          <t>MESMEN001</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="n">
+        <v>1213928</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="41" t="inlineStr">
         <is>
+          <t>INMMSPRET1</t>
+        </is>
+      </c>
+      <c r="B30" s="42" t="n">
+        <v>785885</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="41" t="inlineStr">
+        <is>
+          <t>INPPREVIND</t>
+        </is>
+      </c>
+      <c r="B31" s="42" t="n">
+        <v>691892</v>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="40" t="inlineStr">
+        <is>
+          <t>Fidélité par tranche d'âge</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="41" t="inlineStr">
+        <is>
+          <t>Tranche la plus fidèle</t>
+        </is>
+      </c>
+      <c r="B34" s="50" t="inlineStr">
+        <is>
+          <t>Plus de 80 ans</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="41" t="inlineStr">
+        <is>
           <t>Taux radiation</t>
         </is>
       </c>
-      <c r="B30" s="43" t="n">
+      <c r="B35" s="43" t="n">
         <v>0.0002279454624199341</v>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" s="40" t="inlineStr">
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="40" t="inlineStr">
         <is>
           <t>Par type assuré</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="44" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="44" t="inlineStr">
         <is>
           <t>Type assuré</t>
         </is>
       </c>
-      <c r="B33" s="44" t="inlineStr">
+      <c r="B38" s="44" t="inlineStr">
         <is>
           <t>pp non radiés</t>
         </is>
       </c>
-      <c r="C33" s="44" t="inlineStr">
+      <c r="C38" s="44" t="inlineStr">
         <is>
           <t>% total</t>
         </is>
       </c>
-      <c r="D33" s="44" t="inlineStr">
+      <c r="D38" s="44" t="inlineStr">
         <is>
           <t>Taux radiation</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="51" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="51" t="inlineStr">
         <is>
           <t>ASSURE</t>
         </is>
       </c>
-      <c r="B34" s="45" t="n">
+      <c r="B39" s="45" t="n">
         <v>3203817</v>
       </c>
-      <c r="C34" s="52" t="n">
+      <c r="C39" s="52" t="n">
         <v>0.7812230936299615</v>
       </c>
-      <c r="D34" s="52" t="n">
+      <c r="D39" s="52" t="n">
         <v>0.002950855183051966</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="51" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="51" t="inlineStr">
         <is>
           <t>ENFANT</t>
         </is>
       </c>
-      <c r="B35" s="45" t="n">
+      <c r="B40" s="45" t="n">
         <v>685155</v>
       </c>
-      <c r="C35" s="52" t="n">
+      <c r="C40" s="52" t="n">
         <v>0.1670691268309133</v>
       </c>
-      <c r="D35" s="52" t="n">
+      <c r="D40" s="52" t="n">
         <v>0.006480285482846947</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="51" t="inlineStr">
-        <is>
-          <t>CONJOI</t>
-        </is>
-      </c>
-      <c r="B36" s="45" t="n">
-        <v>212038</v>
-      </c>
-      <c r="C36" s="52" t="n">
-        <v>0.05170363423600966</v>
-      </c>
-      <c r="D36" s="52" t="n">
-        <v>0.004777445552212339</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="51" t="inlineStr">
-        <is>
-          <t>ASCEND</t>
-        </is>
-      </c>
-      <c r="B37" s="45" t="n">
-        <v>17</v>
-      </c>
-      <c r="C37" s="52" t="n">
-        <v>4.145303115536669e-06</v>
-      </c>
-      <c r="D37" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38"/>
-    <row r="39">
-      <c r="A39" s="40" t="inlineStr">
-        <is>
-          <t>Par société</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="44" t="inlineStr">
-        <is>
-          <t>Société</t>
-        </is>
-      </c>
-      <c r="B40" s="44" t="inlineStr">
-        <is>
-          <t>pp non radiés</t>
-        </is>
-      </c>
-      <c r="C40" s="44" t="inlineStr">
-        <is>
-          <t>% total</t>
-        </is>
-      </c>
-      <c r="D40" s="44" t="inlineStr">
-        <is>
-          <t>Taux radiation</t>
-        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="51" t="inlineStr">
         <is>
-          <t>010</t>
+          <t>CONJOI</t>
         </is>
       </c>
       <c r="B41" s="45" t="n">
-        <v>4061007</v>
+        <v>212038</v>
       </c>
       <c r="C41" s="52" t="n">
-        <v>0.9902414687833072</v>
+        <v>0.05170363423600966</v>
       </c>
       <c r="D41" s="52" t="n">
-        <v>0.003288100709996314</v>
+        <v>0.004777445552212339</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="51" t="inlineStr">
         <is>
+          <t>ASCEND</t>
+        </is>
+      </c>
+      <c r="B42" s="45" t="n">
+        <v>17</v>
+      </c>
+      <c r="C42" s="52" t="n">
+        <v>4.145303115536669e-06</v>
+      </c>
+      <c r="D42" s="52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="40" t="inlineStr">
+        <is>
+          <t>Par société</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="44" t="inlineStr">
+        <is>
+          <t>Société</t>
+        </is>
+      </c>
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>pp non radiés</t>
+        </is>
+      </c>
+      <c r="C45" s="44" t="inlineStr">
+        <is>
+          <t>% total</t>
+        </is>
+      </c>
+      <c r="D45" s="44" t="inlineStr">
+        <is>
+          <t>Taux radiation</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="51" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="B46" s="45" t="n">
+        <v>4061007</v>
+      </c>
+      <c r="C46" s="52" t="n">
+        <v>0.9902414687833072</v>
+      </c>
+      <c r="D46" s="52" t="n">
+        <v>0.003288100709996314</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="51" t="inlineStr">
+        <is>
           <t>044</t>
         </is>
       </c>
-      <c r="B42" s="45" t="n">
+      <c r="B47" s="45" t="n">
         <v>30575</v>
       </c>
-      <c r="C42" s="52" t="n">
+      <c r="C47" s="52" t="n">
         <v>0.007455449573972569</v>
       </c>
-      <c r="D42" s="52" t="n">
+      <c r="D47" s="52" t="n">
         <v>0.04994276369582993</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="51" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="51" t="inlineStr">
         <is>
           <t>052</t>
         </is>
       </c>
-      <c r="B43" s="45" t="n">
+      <c r="B48" s="45" t="n">
         <v>8631</v>
       </c>
-      <c r="C43" s="52" t="n">
+      <c r="C48" s="52" t="n">
         <v>0.002104594775893941</v>
       </c>
-      <c r="D43" s="52" t="n">
+      <c r="D48" s="52" t="n">
         <v>0.0016220600162206</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="51" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="51" t="inlineStr">
         <is>
           <t>073</t>
         </is>
       </c>
-      <c r="B44" s="45" t="n">
+      <c r="B49" s="45" t="n">
         <v>814</v>
       </c>
-      <c r="C44" s="52" t="n">
+      <c r="C49" s="52" t="n">
         <v>0.0001984868668262852</v>
       </c>
-      <c r="D44" s="52" t="n">
+      <c r="D49" s="52" t="n">
         <v>0.01597051597051597</v>
       </c>
     </row>

</xml_diff>